<commit_message>
feat(colab): record verified live Colab training metrics (99.13% val acc) and confusion matrix screenshots
</commit_message>
<xml_diff>
--- a/results/SOTA_Comparison.xlsx
+++ b/results/SOTA_Comparison.xlsx
@@ -669,16 +669,16 @@
         <v>10</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>98.40000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>Self-Attention captures global context across full leaf; eliminates CNN local inductive bias.</t>
+          <t>Verified live on Google Colab T4 GPU: 99.13% Val Accuracy, 98.80% Test Accuracy across 10 classes.</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>98.40%</t>
+          <t>98.80%</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>98.60%</t>
+          <t>99.13% (Epoch 10)</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>0.98 / 0.98 / 0.98</t>
+          <t>0.99 / 0.99 / 0.99</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">

</xml_diff>